<commit_message>
4 factors C alternative included
</commit_message>
<xml_diff>
--- a/phase3-validation/06_alternative-structures/output/EFA_Summary_Consolidated.xlsx
+++ b/phase3-validation/06_alternative-structures/output/EFA_Summary_Consolidated.xlsx
@@ -8783,10 +8783,10 @@
         <v>39</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9019</v>
+        <v>0.9018</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9019</v>
+        <v>0.9018</v>
       </c>
       <c r="E2" t="n">
         <v>-0.1003</v>
@@ -9110,7 +9110,7 @@
         <v>0.5926</v>
       </c>
       <c r="H14" t="n">
-        <v>1.5983</v>
+        <v>1.5982</v>
       </c>
     </row>
   </sheetData>
@@ -9248,10 +9248,10 @@
         <v>39</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7003</v>
+        <v>0.7002</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7003</v>
+        <v>0.7002</v>
       </c>
       <c r="E5" t="n">
         <v>0.0946</v>
@@ -9463,10 +9463,10 @@
         <v>1.0141</v>
       </c>
       <c r="G12" t="n">
-        <v>0.9327</v>
+        <v>0.9326</v>
       </c>
       <c r="H12" t="n">
-        <v>0.0673</v>
+        <v>0.0674</v>
       </c>
       <c r="I12" t="n">
         <v>1.0145</v>
@@ -9645,10 +9645,10 @@
         <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7284</v>
+        <v>0.7283</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7284</v>
+        <v>0.7283</v>
       </c>
       <c r="E4" t="n">
         <v>0.0559</v>
@@ -9837,13 +9837,13 @@
         <v>56</v>
       </c>
       <c r="C10" t="n">
-        <v>0.5351</v>
+        <v>0.535</v>
       </c>
       <c r="D10" t="n">
         <v>0.0722</v>
       </c>
       <c r="E10" t="n">
-        <v>0.5351</v>
+        <v>0.535</v>
       </c>
       <c r="F10" t="n">
         <v>0.1908</v>
@@ -9858,7 +9858,7 @@
         <v>0.4581</v>
       </c>
       <c r="J10" t="n">
-        <v>1.3663</v>
+        <v>1.3664</v>
       </c>
     </row>
     <row r="11">

</xml_diff>